<commit_message>
Fix ELAR IMDI export for imported multilingual slash syntax
Honor virtual multilingual slash-syntax values during IMDI export so ELAR metadata exported from spreadsheet import no longer depends on a user clicking each field first.

Route generic multilingual field export and comma-separated topic/keyword key export through metadata-language slot order, preserving existing tagged multilingual behavior while covering imported slash-syntax data.

Add regression coverage for slash-syntax field export, keyword export, and topic export, and document the new export-side compatibility logic with targeted comments.
</commit_message>
<xml_diff>
--- a/sample data/LingMetaX_Sessions.xlsx
+++ b/sample data/LingMetaX_Sessions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\lameta\sample data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448AA796-D2FB-490B-9AB8-9EB6B126C973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5482F98-B373-4B44-8BEE-186C5E318C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25155" yWindow="765" windowWidth="21600" windowHeight="12735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="6360" windowWidth="28110" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -165,9 +168,6 @@
     <t>Author</t>
   </si>
   <si>
-    <t>Normal</t>
-  </si>
-  <si>
     <t>without date</t>
   </si>
   <si>
@@ -507,6 +507,9 @@
   </si>
   <si>
     <t>hɛˈləʊ wɜːld</t>
+  </si>
+  <si>
+    <t>Normal / Título normal</t>
   </si>
 </sst>
 </file>
@@ -879,32 +882,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AQ7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" customWidth="1"/>
-    <col min="16" max="16" width="27.42578125" customWidth="1"/>
-    <col min="17" max="17" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.453125" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.26953125" customWidth="1"/>
+    <col min="5" max="5" width="16.7265625" customWidth="1"/>
+    <col min="6" max="6" width="15.7265625" customWidth="1"/>
+    <col min="8" max="8" width="14.1796875" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" customWidth="1"/>
+    <col min="10" max="10" width="15.453125" customWidth="1"/>
+    <col min="11" max="11" width="19.81640625" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" customWidth="1"/>
+    <col min="14" max="14" width="9.1796875" customWidth="1"/>
+    <col min="16" max="16" width="27.453125" customWidth="1"/>
+    <col min="17" max="17" width="21.1796875" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
-    <col min="33" max="33" width="17.7109375" customWidth="1"/>
-    <col min="34" max="34" width="30.140625" customWidth="1"/>
-    <col min="35" max="35" width="19.42578125" customWidth="1"/>
-    <col min="36" max="36" width="21.140625" customWidth="1"/>
+    <col min="33" max="33" width="17.7265625" customWidth="1"/>
+    <col min="34" max="34" width="30.1796875" customWidth="1"/>
+    <col min="35" max="35" width="19.453125" customWidth="1"/>
+    <col min="36" max="36" width="21.1796875" customWidth="1"/>
     <col min="40" max="40" width="18" customWidth="1"/>
-    <col min="42" max="42" width="17.42578125" customWidth="1"/>
+    <col min="42" max="42" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1032,167 +1035,167 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" ht="16" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>44367</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
         <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
         <v>67</v>
       </c>
-      <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>68</v>
-      </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="K2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" t="s">
         <v>75</v>
       </c>
-      <c r="K2" t="s">
-        <v>77</v>
-      </c>
-      <c r="L2" t="s">
-        <v>76</v>
-      </c>
       <c r="M2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="W2" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD2" t="s">
         <v>58</v>
       </c>
-      <c r="W2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>59</v>
-      </c>
       <c r="AH2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI2" t="s">
         <v>44</v>
       </c>
       <c r="AJ2" t="s">
+        <v>50</v>
+      </c>
+      <c r="AL2" t="s">
         <v>51</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AN2" t="s">
         <v>52</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AP2" t="s">
         <v>53</v>
       </c>
-      <c r="AP2" t="s">
-        <v>54</v>
-      </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" t="s">
-        <v>74</v>
-      </c>
       <c r="L3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AH3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>44084</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" t="s">
-        <v>71</v>
-      </c>
       <c r="K4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AH4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AI4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>44085</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AI5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>44086</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
         <v>80</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>81</v>
-      </c>
-      <c r="C7" t="s">
-        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>